<commit_message>
Add tag-based question filtering: tags management, per-question tags, exam pool filter, bulk import auto-create tags
</commit_message>
<xml_diff>
--- a/public/questions-template.xlsx
+++ b/public/questions-template.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="29">
   <si>
     <t>title</t>
   </si>
@@ -39,6 +39,9 @@
     <t>reference_solution</t>
   </si>
   <si>
+    <t>tags</t>
+  </si>
+  <si>
     <t>test_cases</t>
   </si>
   <si>
@@ -48,24 +51,23 @@
     <t>easy</t>
   </si>
   <si>
-    <t>Diberikan sebuah bilangan bulat **n**, hitung nilai kuadratnya.
-**Contoh:**
-- Input: `5`
-- Output: `25`</t>
+    <t>Diberikan sebuah bilangan bulat n, hitung nilai kuadratnya.</t>
   </si>
   <si>
     <t>n = int(input())
 # Tulis kode di bawah ini</t>
   </si>
   <si>
-    <t>Gunakan operator perkalian `*`.
-Kuadrat = n x n.</t>
+    <t>Gunakan operator perkalian *.</t>
   </si>
   <si>
     <t>n = int(input())
 print(n * n)</t>
   </si>
   <si>
+    <t>matematika,loop</t>
+  </si>
+  <si>
     <t>5||25||0;-3||9||1;0||0||0</t>
   </si>
   <si>
@@ -81,33 +83,30 @@
     <t>Yes</t>
   </si>
   <si>
-    <t>Question title, max 255 characters</t>
-  </si>
-  <si>
-    <t>Must be: easy, medium, or hard</t>
-  </si>
-  <si>
-    <t>Markdown supported. LaTeX: $$...$$ Diagram: ```mermaid</t>
-  </si>
-  <si>
-    <t>Numeric score weight (e.g. 10, 20.5)</t>
+    <t>Max 255 chars</t>
+  </si>
+  <si>
+    <t>easy / medium / hard</t>
+  </si>
+  <si>
+    <t>Markdown supported</t>
+  </si>
+  <si>
+    <t>Angka, misal 10 atau 20.5</t>
   </si>
   <si>
     <t>No</t>
   </si>
   <si>
-    <t>Starter code shown to students. Leave blank if none.</t>
-  </si>
-  <si>
-    <t>Hint shown when student requests. Leave blank if none.</t>
-  </si>
-  <si>
-    <t>Correct solution for admin reference. Leave blank if none.</t>
+    <t>Boleh kosong</t>
+  </si>
+  <si>
+    <t>Nama tag pisah koma, misal: array,loop,sorting. Auto-create jika belum ada.</t>
   </si>
   <si>
     <t>Format: input||expected_output||is_hidden(0/1)
-Multiple test cases separated by semicolon ;
-Example: 5||25||0;-3||9||1</t>
+Pisah pakai ;
+Contoh: 5||25||0;-3||9||1</t>
   </si>
 </sst>
 </file>
@@ -482,7 +481,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="true" style="0"/>
@@ -492,10 +491,11 @@
     <col min="5" max="5" width="40" customWidth="true" style="3"/>
     <col min="6" max="6" width="40" customWidth="true" style="3"/>
     <col min="7" max="7" width="40" customWidth="true" style="3"/>
-    <col min="8" max="8" width="50" customWidth="true" style="0"/>
+    <col min="8" max="8" width="30" customWidth="true" style="0"/>
+    <col min="9" max="9" width="50" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -520,31 +520,37 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" customHeight="1" ht="80">
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" customHeight="1" ht="60">
       <c r="A2" s="4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" s="5">
         <v>20</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -559,7 +565,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="true" style="0"/>
@@ -569,13 +575,13 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -583,10 +589,10 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -594,10 +600,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -605,10 +611,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -616,10 +622,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -627,10 +633,10 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -638,10 +644,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -649,7 +655,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>26</v>
@@ -660,10 +666,21 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update bulk import Excel template for all question types
</commit_message>
<xml_diff>
--- a/public/questions-template.xlsx
+++ b/public/questions-template.xlsx
@@ -4,11 +4,11 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
+    <workbookView activeTab="1" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
     <sheet name="Questions" sheetId="1" r:id="rId4"/>
-    <sheet name="Notes" sheetId="2" r:id="rId5"/>
+    <sheet name="Instructions" sheetId="2" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
@@ -16,11 +16,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="91">
   <si>
     <t>title</t>
   </si>
   <si>
+    <t>type</t>
+  </si>
+  <si>
     <t>difficulty</t>
   </si>
   <si>
@@ -45,68 +48,250 @@
     <t>test_cases</t>
   </si>
   <si>
-    <t>Kuadrat Sebuah Angka</t>
+    <t>options</t>
+  </si>
+  <si>
+    <t>fill_blank_answer</t>
+  </si>
+  <si>
+    <t>true_false_answer</t>
+  </si>
+  <si>
+    <t>language</t>
+  </si>
+  <si>
+    <t>Sum of Two Numbers</t>
+  </si>
+  <si>
+    <t>coding</t>
   </si>
   <si>
     <t>easy</t>
   </si>
   <si>
-    <t>Diberikan sebuah bilangan bulat n, hitung nilai kuadratnya.</t>
-  </si>
-  <si>
-    <t>n = int(input())
-# Tulis kode di bawah ini</t>
-  </si>
-  <si>
-    <t>Gunakan operator perkalian *.</t>
-  </si>
-  <si>
-    <t>n = int(input())
-print(n * n)</t>
-  </si>
-  <si>
-    <t>matematika,loop</t>
-  </si>
-  <si>
-    <t>5||25||0;-3||9||1;0||0||0</t>
+    <t>Write a function that returns the sum of two integers a and b.</t>
+  </si>
+  <si>
+    <t>def solution(a, b):
+    # your code here
+    pass</t>
+  </si>
+  <si>
+    <t>Think about the + operator.</t>
+  </si>
+  <si>
+    <t>def solution(a, b):
+    return a + b</t>
+  </si>
+  <si>
+    <t>math,basics</t>
+  </si>
+  <si>
+    <t>1 2||3||0;-5 10||5||0;0 0||0||1</t>
+  </si>
+  <si>
+    <t>Python (3.8.1)</t>
+  </si>
+  <si>
+    <t>What is the capital of France?</t>
+  </si>
+  <si>
+    <t>multiple_choice</t>
+  </si>
+  <si>
+    <t>Choose the correct capital city of France.</t>
+  </si>
+  <si>
+    <t>The answer is Paris.</t>
+  </si>
+  <si>
+    <t>geography</t>
+  </si>
+  <si>
+    <t>London|*Paris|Berlin|Madrid</t>
+  </si>
+  <si>
+    <t>Which are programming languages?</t>
+  </si>
+  <si>
+    <t>multiple_select</t>
+  </si>
+  <si>
+    <t>Select all items that are programming languages.</t>
+  </si>
+  <si>
+    <t>Python and Java are programming languages.</t>
+  </si>
+  <si>
+    <t>basics</t>
+  </si>
+  <si>
+    <t>*Python|HTML|*Java|CSS</t>
+  </si>
+  <si>
+    <t>Is Python interpreted?</t>
+  </si>
+  <si>
+    <t>true_false</t>
+  </si>
+  <si>
+    <t>True or False: Python is an interpreted language.</t>
+  </si>
+  <si>
+    <t>Python is indeed interpreted.</t>
+  </si>
+  <si>
+    <t>python</t>
+  </si>
+  <si>
+    <t>true</t>
+  </si>
+  <si>
+    <t>Python list append</t>
+  </si>
+  <si>
+    <t>fill_in_blank</t>
+  </si>
+  <si>
+    <t>What method do you use to add an element to the end of a Python list?</t>
+  </si>
+  <si>
+    <t>Think about the opposite of pop.</t>
+  </si>
+  <si>
+    <t>list.append(element)</t>
+  </si>
+  <si>
+    <t>python,basics</t>
+  </si>
+  <si>
+    <t>append</t>
+  </si>
+  <si>
+    <t>Explain OOP principles</t>
+  </si>
+  <si>
+    <t>essay</t>
+  </si>
+  <si>
+    <t>medium</t>
+  </si>
+  <si>
+    <t>Explain the four main principles of Object-Oriented Programming.</t>
+  </si>
+  <si>
+    <t>Encapsulation, Inheritance, Polymorphism, Abstraction.</t>
+  </si>
+  <si>
+    <t>oop,concepts</t>
   </si>
   <si>
     <t>Column</t>
   </si>
   <si>
-    <t>Required</t>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>Required for</t>
   </si>
   <si>
     <t>Notes</t>
   </si>
   <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>Max 255 chars</t>
-  </si>
-  <si>
-    <t>easy / medium / hard</t>
-  </si>
-  <si>
-    <t>Markdown supported</t>
-  </si>
-  <si>
-    <t>Angka, misal 10 atau 20.5</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Boleh kosong</t>
-  </si>
-  <si>
-    <t>Nama tag pisah koma, misal: array,loop,sorting. Auto-create jika belum ada.</t>
-  </si>
-  <si>
-    <t>Format: input||expected_output||is_hidden(0/1)
-Pisah pakai ;
-Contoh: 5||25||0;-3||9||1</t>
+    <t>A</t>
+  </si>
+  <si>
+    <t>All</t>
+  </si>
+  <si>
+    <t>Question title (max 255 chars)</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>coding | multiple_choice | multiple_select | true_false | fill_in_blank | essay</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>easy | medium | hard</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>Question body. Markdown supported.</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>Number (e.g. 10)</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>coding (optional)</t>
+  </si>
+  <si>
+    <t>Code shown to student at start</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
+  <si>
+    <t>Optional</t>
+  </si>
+  <si>
+    <t>Markdown. Shown when student requests hint.</t>
+  </si>
+  <si>
+    <t>H</t>
+  </si>
+  <si>
+    <t>Admin-only reference. Not shown to students.</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>Comma-separated tag names. e.g. math,loops</t>
+  </si>
+  <si>
+    <t>J</t>
+  </si>
+  <si>
+    <t>Semicolon-separated. Format: input||output||hidden(0/1). e.g. 2 3||5||0;0 0||0||1</t>
+  </si>
+  <si>
+    <t>K</t>
+  </si>
+  <si>
+    <t>multiple_choice, multiple_select</t>
+  </si>
+  <si>
+    <t>Pipe-separated. Prefix correct option(s) with *. e.g. Option A|*Correct B|Option C</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>The exact correct answer (compared case-insensitively)</t>
+  </si>
+  <si>
+    <t>M</t>
+  </si>
+  <si>
+    <t>true or false (or 1 / 0)</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>Judge0 language name. Falls back to import default if empty.</t>
   </si>
 </sst>
 </file>
@@ -134,7 +319,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -149,12 +334,42 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF0F4FF"/>
+        <fgColor rgb="FFEEF2FF"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF0FDF4"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF7ED"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFDF4FF"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFBEB"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF1F2"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -162,23 +377,64 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF818CF8"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF818CF8"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF818CF8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF818CF8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFE2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
       <alignment vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="3" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="3" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="3" borderId="2" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="4" borderId="2" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="5" borderId="2" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="6" borderId="2" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="7" borderId="2" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="8" borderId="2" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0"/>
@@ -481,40 +737,45 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="true" style="0"/>
-    <col min="2" max="2" width="12" customWidth="true" style="0"/>
-    <col min="3" max="3" width="60" customWidth="true" style="3"/>
-    <col min="4" max="4" width="16" customWidth="true" style="3"/>
-    <col min="5" max="5" width="40" customWidth="true" style="3"/>
-    <col min="6" max="6" width="40" customWidth="true" style="3"/>
-    <col min="7" max="7" width="40" customWidth="true" style="3"/>
+    <col min="2" max="2" width="18" customWidth="true" style="0"/>
+    <col min="3" max="3" width="12" customWidth="true" style="0"/>
+    <col min="4" max="4" width="45" customWidth="true" style="0"/>
+    <col min="5" max="5" width="14" customWidth="true" style="0"/>
+    <col min="6" max="6" width="30" customWidth="true" style="0"/>
+    <col min="7" max="7" width="25" customWidth="true" style="0"/>
     <col min="8" max="8" width="30" customWidth="true" style="0"/>
-    <col min="9" max="9" width="50" customWidth="true" style="0"/>
+    <col min="9" max="9" width="20" customWidth="true" style="0"/>
+    <col min="10" max="10" width="40" customWidth="true" style="0"/>
+    <col min="11" max="11" width="40" customWidth="true" style="0"/>
+    <col min="12" max="12" width="20" customWidth="true" style="0"/>
+    <col min="13" max="13" width="16" customWidth="true" style="0"/>
+    <col min="14" max="14" width="22" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:14" customHeight="1" ht="22">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
@@ -523,35 +784,219 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" customHeight="1" ht="60">
-      <c r="A2" s="4" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="5">
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" customHeight="1" ht="50">
+      <c r="A2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" s="3">
+        <v>10</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H2" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="E2" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" customHeight="1" ht="50">
+      <c r="A3" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>16</v>
       </c>
+      <c r="D3" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" s="4">
+        <v>5</v>
+      </c>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+    </row>
+    <row r="4" spans="1:14" customHeight="1" ht="50">
+      <c r="A4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4" s="5">
+        <v>5</v>
+      </c>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="J4" s="5"/>
+      <c r="K4" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="L4" s="5"/>
+      <c r="M4" s="5"/>
+      <c r="N4" s="5"/>
+    </row>
+    <row r="5" spans="1:14" customHeight="1" ht="50">
+      <c r="A5" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" s="6">
+        <v>5</v>
+      </c>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
+      <c r="L5" s="6"/>
+      <c r="M5" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="N5" s="6"/>
+    </row>
+    <row r="6" spans="1:14" customHeight="1" ht="50">
+      <c r="A6" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E6" s="7">
+        <v>5</v>
+      </c>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="J6" s="7"/>
+      <c r="K6" s="7"/>
+      <c r="L6" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="M6" s="7"/>
+      <c r="N6" s="7"/>
+    </row>
+    <row r="7" spans="1:14" customHeight="1" ht="50">
+      <c r="A7" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E7" s="8">
+        <v>20</v>
+      </c>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="I7" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
     </row>
   </sheetData>
   <printOptions gridLines="false" gridLinesSet="true"/>
@@ -565,122 +1010,223 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="true" style="0"/>
-    <col min="2" max="2" width="10" customWidth="true" style="0"/>
-    <col min="3" max="3" width="70" customWidth="true" style="0"/>
+    <col min="1" max="1" width="8" customWidth="true" style="0"/>
+    <col min="2" max="2" width="20" customWidth="true" style="0"/>
+    <col min="3" max="3" width="30" customWidth="true" style="0"/>
+    <col min="4" max="4" width="80" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
+    <row r="1" spans="1:4">
+      <c r="A1" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
+      <c r="C2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
+      <c r="C3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
       <c r="A4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
+      <c r="C4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
       <c r="A5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
+      <c r="C5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
       <c r="A6" t="s">
+        <v>68</v>
+      </c>
+      <c r="B6" t="s">
         <v>4</v>
       </c>
-      <c r="B6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
+      <c r="C6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
       <c r="A7" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" t="s">
         <v>5</v>
       </c>
-      <c r="B7" t="s">
-        <v>25</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
+      <c r="C7" t="s">
+        <v>71</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
       <c r="A8" t="s">
+        <v>73</v>
+      </c>
+      <c r="B8" t="s">
         <v>6</v>
       </c>
-      <c r="B8" t="s">
-        <v>25</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
+      <c r="C8" t="s">
+        <v>74</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
       <c r="A9" t="s">
+        <v>76</v>
+      </c>
+      <c r="B9" t="s">
         <v>7</v>
       </c>
-      <c r="B9" t="s">
-        <v>25</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
+      <c r="C9" t="s">
+        <v>74</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
       <c r="A10" t="s">
+        <v>78</v>
+      </c>
+      <c r="B10" t="s">
         <v>8</v>
       </c>
-      <c r="B10" t="s">
-        <v>20</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>28</v>
+      <c r="C10" t="s">
+        <v>74</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" t="s">
+        <v>80</v>
+      </c>
+      <c r="B11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" t="s">
+        <v>82</v>
+      </c>
+      <c r="B12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12" t="s">
+        <v>83</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" t="s">
+        <v>85</v>
+      </c>
+      <c r="B13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" t="s">
+        <v>87</v>
+      </c>
+      <c r="B14" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" t="s">
+        <v>37</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" t="s">
+        <v>89</v>
+      </c>
+      <c r="B15" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" t="s">
+        <v>71</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>